<commit_message>
fix: auto timesheet log
</commit_message>
<xml_diff>
--- a/test_data/template_staff_info.xlsx
+++ b/test_data/template_staff_info.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t xml:space="preserve">stt</t>
   </si>
@@ -92,6 +92,18 @@
   </si>
   <si>
     <t xml:space="preserve">VTN-CUONGLH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyễn Hoàng Việt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vietnh41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.221.2.91</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VTN-VIETNH41</t>
   </si>
 </sst>
 </file>
@@ -202,7 +214,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -217,6 +229,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -296,8 +312,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
@@ -400,6 +416,29 @@
         <v>23</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>293048</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>